<commit_message>
docs: restrict AgentTrace to two read-only detection findings
</commit_message>
<xml_diff>
--- a/outputs/01a180d7-4423-7a82-bd37-7dbc25ea89ba/AgentTrace_Capabilities_and_Limits.xlsx
+++ b/outputs/01a180d7-4423-7a82-bd37-7dbc25ea89ba/AgentTrace_Capabilities_and_Limits.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent detection" sheetId="1" r:id="Ra88eacdd9bc34466"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content detection" sheetId="2" r:id="R634ea1f4bc924d37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client standards" sheetId="3" r:id="R5b8e293e46024334"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent detection" sheetId="1" r:id="R5ae383d7a4cc4769"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content detection" sheetId="2" r:id="R7ff99ae56e734dec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client standards" sheetId="3" r:id="R5c293025c4dd4d08"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -229,7 +229,337 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="15">
+  <x:dxfs count="45">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF215B3C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE5F1E9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF79500F"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF1D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8C283B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFBE7EA"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8C283B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFBE7EA"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE9EDF3"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF215B3C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE5F1E9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF79500F"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF1D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8C283B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFBE7EA"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8C283B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFBE7EA"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE9EDF3"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF215B3C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE5F1E9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF79500F"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF1D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8C283B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFBE7EA"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8C283B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFBE7EA"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE9EDF3"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF215B3C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE5F1E9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF79500F"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF1D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8C283B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFBE7EA"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8C283B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFBE7EA"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE9EDF3"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF215B3C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE5F1E9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF79500F"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF1D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8C283B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFBE7EA"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8C283B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFBE7EA"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE9EDF3"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF215B3C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE5F1E9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF79500F"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF1D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8C283B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFBE7EA"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8C283B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFBE7EA"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE9EDF3"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
@@ -703,7 +1033,7 @@
     </x:row>
     <x:row r="6" ht="22" customHeight="1">
       <x:c r="A6" s="13" t="str">
-        <x:v>Filter by feasibility. Read the conditions before making a client commitment. Definitions are on Client standards.</x:v>
+        <x:v>Detection only: AgentTrace reads evidence and flags findings. It does not draft, send, approve or automate email.</x:v>
       </x:c>
       <x:c r="B6" s="12"/>
       <x:c r="C6" s="12"/>
@@ -736,87 +1066,87 @@
     </x:row>
     <x:row r="9" ht="64" customHeight="1">
       <x:c r="A9" s="23" t="str">
-        <x:v>Agent sends through a monitored workflow</x:v>
+        <x:v>Email sent by an agent in an existing monitored system</x:v>
       </x:c>
       <x:c r="B9" s="23" t="str">
         <x:v>Possible with evidence</x:v>
       </x:c>
       <x:c r="C9" s="21" t="str">
-        <x:v>Verify that a known agent executed the send and link it to the specific email.</x:v>
+        <x:v>Flag the email as agent-sent when existing execution evidence reliably matches the sent message.</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
-        <x:v>Needs trusted execution records and a matching sent-message observation. An app name alone is not enough.</x:v>
+        <x:v>Requires trusted source records. AgentTrace reads them and never executes the source agent or send.</x:v>
       </x:c>
       <x:c r="E9" s="21" t="str">
-        <x:v>An integrated assistant sends an invoice email and its execution record matches that message.</x:v>
+        <x:v>An existing assistant sends an invoice email. AgentTrace detects its origin from available records.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="64" customHeight="1">
       <x:c r="A10" s="24" t="str">
-        <x:v>Agent sends after a person approves</x:v>
+        <x:v>Email sent by an agent after external human approval</x:v>
       </x:c>
       <x:c r="B10" s="24" t="str">
         <x:v>Possible with evidence</x:v>
       </x:c>
       <x:c r="C10" s="22" t="str">
-        <x:v>Record the agent send and the recorded human approval as separate facts.</x:v>
+        <x:v>Flag as agent-sent when reliable send evidence exists. External approval does not change that finding.</x:v>
       </x:c>
       <x:c r="D10" s="22" t="str">
-        <x:v>Approval must match the exact message and recipients. It does not remove agent involvement.</x:v>
+        <x:v>Approval happens outside AgentTrace. The product has no approval requests, queues or approval screens.</x:v>
       </x:c>
       <x:c r="E10" s="22" t="str">
-        <x:v>A person approves the draft. The agent then sends it: approved agent send.</x:v>
+        <x:v>A person approves in another tool. An agent sends. AgentTrace flags the already-sent email.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="64" customHeight="1">
       <x:c r="A11" s="23" t="str">
-        <x:v>Agent sends without per-message approval</x:v>
+        <x:v>Email sent autonomously by an agent</x:v>
       </x:c>
       <x:c r="B11" s="23" t="str">
         <x:v>Possible with evidence</x:v>
       </x:c>
       <x:c r="C11" s="21" t="str">
-        <x:v>Identify autonomous execution within a fully observed, authorized workflow.</x:v>
+        <x:v>Flag as agent-sent using existing execution and message evidence.</x:v>
       </x:c>
       <x:c r="D11" s="21" t="str">
-        <x:v>Missing approval logs mean unknown. They do not prove that nobody approved the message.</x:v>
+        <x:v>Autonomy is source context, not a separate product output. AgentTrace does not authorize or operate the agent.</x:v>
       </x:c>
       <x:c r="E11" s="21" t="str">
-        <x:v>An agent sends a routine update under standing authorization, with a complete execution trail.</x:v>
+        <x:v>An existing agent sends a routine update. AgentTrace reads the resulting email and available evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="64" customHeight="1">
       <x:c r="A12" s="24" t="str">
-        <x:v>Agent drafts; a person sends</x:v>
+        <x:v>An AI-created draft is sent manually by a person</x:v>
       </x:c>
       <x:c r="B12" s="24" t="str">
         <x:v>Possible with evidence</x:v>
       </x:c>
       <x:c r="C12" s="22" t="str">
-        <x:v>Identify agent participation in drafting while keeping send execution separate.</x:v>
+        <x:v>Do not flag agent sending based on drafting alone. Assess the wording independently for AI content.</x:v>
       </x:c>
       <x:c r="D12" s="22" t="str">
-        <x:v>Drafting evidence is not evidence that the agent clicked or executed Send.</x:v>
+        <x:v>The send action determines the first finding. AI drafting or mailbox reading alone is insufficient.</x:v>
       </x:c>
       <x:c r="E12" s="22" t="str">
-        <x:v>The agent creates the draft. A person sends it: agent involvement, human send observed.</x:v>
+        <x:v>A person sends an assistant-written draft. A content flag may be raised without an agent-sent flag.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="64" customHeight="1">
       <x:c r="A13" s="23" t="str">
-        <x:v>Known non-AI script versus AI agent</x:v>
+        <x:v>An existing non-AI application sends email</x:v>
       </x:c>
       <x:c r="B13" s="23" t="str">
         <x:v>Possible with evidence</x:v>
       </x:c>
       <x:c r="C13" s="21" t="str">
-        <x:v>Distinguish conventional automation when the specific execution path is known.</x:v>
+        <x:v>Avoid an agent-sent flag when evidence establishes a non-AI send. Assess content independently.</x:v>
       </x:c>
       <x:c r="D13" s="21" t="str">
-        <x:v>A shared application or API can run both types. Classify the execution, not just the app.</x:v>
+        <x:v>A shared app can support different execution types. App identity alone does not establish AI sending.</x:v>
       </x:c>
       <x:c r="E13" s="21" t="str">
-        <x:v>A scheduled reporting script sends human-written text: conventional automation.</x:v>
+        <x:v>A reporting script sends human-written text. AgentTrace does not treat automation alone as AI.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="64" customHeight="1">
@@ -827,13 +1157,13 @@
         <x:v>Possible with evidence</x:v>
       </x:c>
       <x:c r="C14" s="22" t="str">
-        <x:v>Name the authenticated application or agent when execution evidence establishes its identity.</x:v>
+        <x:v>Show authenticated application or agent identity as supporting evidence for the agent-sent finding.</x:v>
       </x:c>
       <x:c r="D14" s="22" t="str">
-        <x:v>The From address, display name or unsigned header is not proof of the underlying actor.</x:v>
+        <x:v>The From address, display name or unsigned header cannot establish the actual sending mechanism.</x:v>
       </x:c>
       <x:c r="E14" s="22" t="str">
-        <x:v>Show the registered agent and execution ID, rather than guessing from the sender name.</x:v>
+        <x:v>A detection record cites the source application and execution ID. There is no agent control panel.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="64" customHeight="1">
@@ -895,7 +1225,7 @@
         <x:v>Not reliable from email alone</x:v>
       </x:c>
       <x:c r="C18" s="22" t="str">
-        <x:v>Use additional trusted session instrumentation if it is available and permitted.</x:v>
+        <x:v>Analyze authorized message and session evidence that already exists, and report any attribution gap.</x:v>
       </x:c>
       <x:c r="D18" s="22" t="str">
         <x:v>The resulting email and user account may look the same as a manual send.</x:v>
@@ -940,19 +1270,19 @@
     </x:row>
     <x:row r="21" ht="64" customHeight="1">
       <x:c r="A21" s="23" t="str">
-        <x:v>A recipient-side agent reads an incoming email</x:v>
+        <x:v>A recipient-side assistant reads the email</x:v>
       </x:c>
       <x:c r="B21" s="23" t="str">
         <x:v>Not reliable from email alone</x:v>
       </x:c>
       <x:c r="C21" s="21" t="str">
-        <x:v>Record the recipient-side action only if it is observed.</x:v>
+        <x:v>Do not raise an agent-sent flag merely because an assistant on the receiving side read the email.</x:v>
       </x:c>
       <x:c r="D21" s="21" t="str">
-        <x:v>A recipient using an agent does not establish that the sender used one.</x:v>
+        <x:v>Recipient-side activity does not establish the sending mechanism. It is not another product flag.</x:v>
       </x:c>
       <x:c r="E21" s="21" t="str">
-        <x:v>An inbox assistant summarizes an email. That does not make the original sender an agent.</x:v>
+        <x:v>An inbox assistant summarizes an email. AgentTrace must not infer that an agent sent the original.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="64" customHeight="1">
@@ -1008,25 +1338,25 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="B9:B24">
-    <x:cfRule type="expression" dxfId="0" priority="1">
+    <x:cfRule type="expression" dxfId="30" priority="1">
       <x:formula>$B9="Possible with evidence"</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="1" priority="2">
+    <x:cfRule type="expression" dxfId="31" priority="2">
       <x:formula>$B9="Possible but uncertain"</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="2" priority="3">
+    <x:cfRule type="expression" dxfId="32" priority="3">
       <x:formula>$B9="Not reliable from email alone"</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="3" priority="4">
+    <x:cfRule type="expression" dxfId="33" priority="4">
       <x:formula>$B9="Cannot guarantee"</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="4" priority="5">
+    <x:cfRule type="expression" dxfId="34" priority="5">
       <x:formula>$B9="Outside this POC"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c3b74f356a04cbe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb82bfea020934c85"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1092,7 +1422,7 @@
     </x:row>
     <x:row r="6" ht="22" customHeight="1">
       <x:c r="A6" s="13" t="str">
-        <x:v>Filter by feasibility. Read the conditions before making a client commitment. Definitions are on Client standards.</x:v>
+        <x:v>Detection only: AgentTrace reads evidence and flags findings. It does not draft, send, approve or automate email.</x:v>
       </x:c>
       <x:c r="B6" s="12"/>
       <x:c r="C6" s="12"/>
@@ -1125,19 +1455,19 @@
     </x:row>
     <x:row r="9" ht="64" customHeight="1">
       <x:c r="A9" s="23" t="str">
-        <x:v>AI output is linked to the email by trusted records</x:v>
+        <x:v>Existing trusted records link AI output to the email</x:v>
       </x:c>
       <x:c r="B9" s="23" t="str">
         <x:v>Possible with evidence</x:v>
       </x:c>
       <x:c r="C9" s="21" t="str">
-        <x:v>Verify that identified email regions contain output from a trusted generation workflow.</x:v>
+        <x:v>Detect included AI-generated material using existing authorized generation and message-inclusion records.</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
-        <x:v>Needs both generation evidence and trustworthy inclusion history. An output log or hash alone is insufficient.</x:v>
+        <x:v>AgentTrace reads evidence. It does not generate text, insert drafts or provide a generation workflow.</x:v>
       </x:c>
       <x:c r="E9" s="21" t="str">
-        <x:v>A managed assistant generates a paragraph and a tracked insertion links it to the sent draft.</x:v>
+        <x:v>An external tool recorded generation and insertion. AgentTrace checks the records against the email.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="64" customHeight="1">
@@ -1397,25 +1727,25 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="B9:B24">
-    <x:cfRule type="expression" dxfId="5" priority="1">
+    <x:cfRule type="expression" dxfId="35" priority="1">
       <x:formula>$B9="Possible with evidence"</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="6" priority="2">
+    <x:cfRule type="expression" dxfId="36" priority="2">
       <x:formula>$B9="Possible but uncertain"</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="7" priority="3">
+    <x:cfRule type="expression" dxfId="37" priority="3">
       <x:formula>$B9="Not reliable from email alone"</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="8" priority="4">
+    <x:cfRule type="expression" dxfId="38" priority="4">
       <x:formula>$B9="Cannot guarantee"</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="9" priority="5">
+    <x:cfRule type="expression" dxfId="39" priority="5">
       <x:formula>$B9="Outside this POC"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1205c1d4a1824cbf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37bd8bd513864adc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1462,7 +1792,7 @@
     </x:row>
     <x:row r="5" ht="22" customHeight="1">
       <x:c r="A5" s="13" t="str">
-        <x:v>Use these definitions and limits consistently when presenting the POC.</x:v>
+        <x:v>Two independent findings: Email sent by an AI agent. Email contains AI-generated content.</x:v>
       </x:c>
       <x:c r="B5" s="12"/>
       <x:c r="C5" s="12"/>
@@ -1485,13 +1815,13 @@
     </x:row>
     <x:row r="8" ht="52" customHeight="1">
       <x:c r="A8" s="23" t="str">
-        <x:v>Separate questions</x:v>
+        <x:v>Detection-only product</x:v>
       </x:c>
       <x:c r="B8" s="21" t="str">
-        <x:v>Agent detection asks who acted in the email workflow. Content detection asks whether the wording contains AI output.</x:v>
+        <x:v>AgentTrace reads authorized email and evidence, then flags two independent findings: agent-sent email and AI-generated content.</x:v>
       </x:c>
       <x:c r="C8" s="21" t="str">
-        <x:v>Always show separate agent and content results.</x:v>
+        <x:v>No email drafting, sending, approval management, agent execution or workflow automation is provided.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="52" customHeight="1">
@@ -1554,10 +1884,10 @@
         <x:v>Verified versus suspected</x:v>
       </x:c>
       <x:c r="B14" s="21" t="str">
-        <x:v>Verified means supported by trustworthy message-linked evidence. Suspected means a validated statistical signal.</x:v>
+        <x:v>Each finding keeps its evidence grade. Verified requires trustworthy message-linked records. Suspected is an inference.</x:v>
       </x:c>
       <x:c r="C14" s="21" t="str">
-        <x:v>A high model score must not be presented as verified origin.</x:v>
+        <x:v>A high content score does not prove an agent sent the email. Neither finding substitutes for the other.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="52" customHeight="1">
@@ -1565,10 +1895,10 @@
         <x:v>Unknown and not evaluated</x:v>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>Unknown means evidence is insufficient. Not evaluated means analysis was outside scope, unavailable or not authorized.</x:v>
+        <x:v>Insufficient evidence, unsupported input or unavailable analysis must remain explicit. These states are not negative findings.</x:v>
       </x:c>
       <x:c r="C15" s="22" t="str">
-        <x:v>Neither status means human, safe or approved.</x:v>
+        <x:v>Display unknown or not evaluated. Do not silently turn missing evidence into a human or no-AI verdict.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="52" customHeight="1">
@@ -1584,13 +1914,13 @@
     </x:row>
     <x:row r="17" ht="52" customHeight="1">
       <x:c r="A17" s="24" t="str">
-        <x:v>Approval policy</x:v>
+        <x:v>Agent sends after approval</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>Human approval and agent activity can both be present. A recorded approval must match the relevant message version.</x:v>
+        <x:v>An externally approved agent send is still an agent-sent email. Approval is a source-system fact, not an AgentTrace function.</x:v>
       </x:c>
       <x:c r="C17" s="22" t="str">
-        <x:v>No approval record does not prove autonomous action.</x:v>
+        <x:v>Detect the sending mechanism. Do not provide approval requests, approval decisions or approval queues.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="52" customHeight="1">
@@ -1631,21 +1961,21 @@
         <x:v>Use of flags</x:v>
       </x:c>
       <x:c r="B21" s="22" t="str">
-        <x:v>Use suspicion for review in the POC. A flag alone does not establish a data leak, policy breach or malicious intent.</x:v>
+        <x:v>Findings are stored and displayed in AgentTrace. Analyst review concerns the detection result, not permission to send email.</x:v>
       </x:c>
       <x:c r="C21" s="22" t="str">
-        <x:v>Do not automatically block email or make disciplinary conclusions from statistical suspicion.</x:v>
+        <x:v>No mail blocking, quarantine, routing, scheduling or automation actions are part of this product.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="52" customHeight="1">
       <x:c r="A22" s="23" t="str">
-        <x:v>Data handling</x:v>
+        <x:v>Read-only data access</x:v>
       </x:c>
       <x:c r="B22" s="21" t="str">
-        <x:v>Process authorized content inside the approved customer boundary. Minimize retention and restrict access.</x:v>
+        <x:v>Read authorized messages and existing evidence inside the approved customer boundary. Minimize retention and restrict access.</x:v>
       </x:c>
       <x:c r="C22" s="21" t="str">
-        <x:v>Do not send sensitive email to public detector demos or consumer AI services.</x:v>
+        <x:v>No mail-send/write permissions or source-agent execution credentials. Do not upload sensitive email to public detectors.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="52" customHeight="1">
@@ -1664,10 +1994,10 @@
         <x:v>Recommended client description</x:v>
       </x:c>
       <x:c r="B24" s="21" t="str">
-        <x:v>AgentTrace is designed to identify evidenced AI-agent activity and assess eligible English email for AI-generated or substantially rewritten content.</x:v>
+        <x:v>AgentTrace is a detection platform that independently flags email sent by an AI agent and email containing AI-generated content.</x:v>
       </x:c>
       <x:c r="C24" s="21" t="str">
-        <x:v>The POC will establish performance and coverage. Verified evidence, statistical suspicion and unknown cases remain distinct.</x:v>
+        <x:v>It reads and analyzes existing email and evidence. Results distinguish verified findings, suspicion and unknowns. It does not automate email.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="22" customHeight="1">
@@ -1710,10 +2040,10 @@
         <x:v>AgentTrace implementation plan</x:v>
       </x:c>
       <x:c r="B30" s="21" t="str">
-        <x:v>Project scope, evidence rules, exclusions and proposed acceptance gates. Revision 88e182f, 28 October 2026.</x:v>
+        <x:v>Detection-only product scope, two findings, excluded execution features and proposed acceptance gates. Updated 28 October 2026.</x:v>
       </x:c>
       <x:c r="C30" s="27" t="str">
-        <x:v>https://github.com/Kkb113/AgentTrace/blob/88e182fdc4ef4f3cde87db180db90e0f07858821/implementation.md</x:v>
+        <x:v>https://github.com/Kkb113/AgentTrace/blob/main/implementation.md</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="63" customHeight="1">
@@ -1773,34 +2103,34 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="A9:A9">
-    <x:cfRule type="expression" dxfId="10" priority="1">
+    <x:cfRule type="expression" dxfId="40" priority="1">
       <x:formula>$A9="Possible with evidence"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="A10:A10">
-    <x:cfRule type="expression" dxfId="11" priority="2">
+    <x:cfRule type="expression" dxfId="41" priority="2">
       <x:formula>$A10="Possible but uncertain"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="A11:A11">
-    <x:cfRule type="expression" dxfId="12" priority="3">
+    <x:cfRule type="expression" dxfId="42" priority="3">
       <x:formula>$A11="Not reliable from email alone"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="A12:A12">
-    <x:cfRule type="expression" dxfId="13" priority="4">
+    <x:cfRule type="expression" dxfId="43" priority="4">
       <x:formula>$A12="Cannot guarantee"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="A13:A13">
-    <x:cfRule type="expression" dxfId="14" priority="5">
+    <x:cfRule type="expression" dxfId="44" priority="5">
       <x:formula>$A13="Outside this POC"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racae92644fa84d78"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0caf51f9120743a1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re82114affbec41d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64412aeb60d94f65"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>